<commit_message>
add: neue Ordner für die Abgabe
</commit_message>
<xml_diff>
--- a/Verbesserungsliste.xlsx
+++ b/Verbesserungsliste.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\neume\Desktop\MCI\Robotik_Projekt\Optimierung-Laboraufgabe-Robotik\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{206CFD37-8F06-43E8-89AD-D745D773B37F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{463E474D-69FF-4C2D-91AC-A96E13E8205C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ToDos" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="523" uniqueCount="215">
   <si>
     <t>Nr.</t>
   </si>
@@ -101,9 +101,6 @@
   </si>
   <si>
     <t>Hannah</t>
-  </si>
-  <si>
-    <t>Plexiglas mit Nieten</t>
   </si>
   <si>
     <t>Abdeckungen</t>
@@ -365,9 +362,6 @@
     <t>Encoder-Signal und Trigger-Signal an der CNV-Karte von IRB...67 prüfen</t>
   </si>
   <si>
-    <t>ENC A+B Signal des SPS_67 Aufbaus kommt noch nicht (EL2521 konfigurieren), Lichtschranke Trigger kommt komischerweise auch nicht -testen</t>
-  </si>
-  <si>
     <t>SPS: LED Grün/Rot konfigurieren und in Profinet einbinden</t>
   </si>
   <si>
@@ -425,9 +419,6 @@
     <t>Kameraturm + Kamera-Halterung drucken, Kamera-Halterung in CAD verstärken, innen weiß lackieren</t>
   </si>
   <si>
-    <t>Sprühdose (Weiß Matt) ist am Aufbau und kann umgesetzt werden</t>
-  </si>
-  <si>
     <t>3D-Druck restliche Teileträger + Montage</t>
   </si>
   <si>
@@ -467,10 +458,6 @@
     <t>SPS Abdeckung von außen, 4 Löcher, 5mm</t>
   </si>
   <si>
-    <t>Gewinde Nieten wurden vollständig gesetzt
---&gt; Plexiglas muss noch geschnitten werden</t>
-  </si>
-  <si>
     <t>Labels außen</t>
   </si>
   <si>
@@ -498,10 +485,6 @@
     <t>Eloxieren inkl Demontage + Montage</t>
   </si>
   <si>
-    <t>Frage ob wirklich eloxieren ? Kontrast schaut aktuell sehr gut aus… sonst zu schwarz !!!
-Hoher Zeitaufwand (gesamte Anlage demontieren)</t>
-  </si>
-  <si>
     <t>Inbetriebnahme</t>
   </si>
   <si>
@@ -571,18 +554,6 @@
     <t>Bereits gedruckt. Mittelteil mit Magneten muss noch getestet werden (alternative geschraubt)</t>
   </si>
   <si>
-    <t>3D Druck</t>
-  </si>
-  <si>
-    <t>Bleche</t>
-  </si>
-  <si>
-    <t>Stecker, Kabel</t>
-  </si>
-  <si>
-    <t>Elektrik</t>
-  </si>
-  <si>
     <t>To-Dos zur Fertigstellung Zweitaufbau</t>
   </si>
   <si>
@@ -629,24 +600,122 @@
   </si>
   <si>
     <t>Erklärung</t>
+  </si>
+  <si>
+    <t>Kabel</t>
+  </si>
+  <si>
+    <t>Verkabelung zweite Cognex Kamera / und allgemein Profinet Kabel, Encoder usw…</t>
+  </si>
+  <si>
+    <t>Teile bestellen (Karten bei Beckhoff)</t>
+  </si>
+  <si>
+    <t>SPS-Halterung nach oben versetzen – Zwischenadapter gedruckt</t>
+  </si>
+  <si>
+    <t>Sprühdose (Weiß Matt) ist am Aufbau und kann umgesetzt werden
+Wenn noch Zeit umsetzen (aber aufjedenfall einstellungen in Cognex Anleitung übernehmen)</t>
   </si>
   <si>
     <t>Misumi für TCP-Spitze, lange Alu-Spitze verwerfen (wird ersetzt durch TeachingSpitze)
 Neue Halterung wurde konzipiert, gedruckt und getestet --&gt; funktioniert 
-Nur Misumi TCP-Spitzen müssen bestellt werden !!!</t>
-  </si>
-  <si>
-    <t>Kabel</t>
-  </si>
-  <si>
-    <t>Verkabelung zweite Cognex Kamera / und allgemein Profinet Kabel, Encoder usw…</t>
+Nur Misumi TCP-Spitzen müssen bestellt werden !!!
+Mail an Benjamin</t>
+  </si>
+  <si>
+    <t>Gewinde Nieten wurden vollständig gesetzt
+--&gt; Plexiglas muss noch geschnitten werden
+wenn noch Zeit</t>
+  </si>
+  <si>
+    <t>Frage ob wirklich eloxieren ? Kontrast schaut aktuell sehr gut aus… sonst zu schwarz !!!
+Hoher Zeitaufwand (gesamte Anlage demontieren)
+Wird wenndann im Sommer umgesetzt</t>
+  </si>
+  <si>
+    <t>Olli fragen, was damit gemeint ist</t>
+  </si>
+  <si>
+    <t>Bauteile (good, not good)</t>
+  </si>
+  <si>
+    <t>Noch kontrollieren bzw. drucken</t>
+  </si>
+  <si>
+    <t>PDF in der Kiste</t>
+  </si>
+  <si>
+    <t>Inhalt der Kiste aufschreiben (standardmäßiger Inhalt)</t>
+  </si>
+  <si>
+    <t>Eine Kiste mit allen Ersatzteilen usw.</t>
+  </si>
+  <si>
+    <t>Rutsche Aufbau</t>
+  </si>
+  <si>
+    <t>Nochmal drucken</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">ENC A+B Signal des SPS_67 Aufbaus kommt noch nicht (EL2521 konfigurieren), Lichtschranke Trigger kommt komischerweise auch nicht -testen
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Parametrierung der Karten passt nicht</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+Gespräch mit Olli: welche Karte und/oder LevelShifter nachbestellt werden muss (welche Kombo funtioniert)
+Tobias Obwechser, Olli, Oskar Online Meeting durchführen, um Problem zu lösen</t>
+    </r>
+  </si>
+  <si>
+    <t>Oliver/Oskar</t>
+  </si>
+  <si>
+    <t>Bestellliste</t>
+  </si>
+  <si>
+    <t>PE Doppelstockklemmen (5x)
+Zahlen Beschriftung 1-9 (einmal die 1)
+Ethernetkabel (1x 30 cm) und (1x 50cm) und (1x 100cm)
+Steckkarten bestellen (Hannah/Oskar klären mit Olli welche Karte)
+Misumi Spitzen (5x)</t>
+  </si>
+  <si>
+    <t>Plexiglas mit Nieten
+Wird nicht mehr umgesetzt (abgesprochen mit Benjamin)</t>
+  </si>
+  <si>
+    <t>Zweite Box ist im Laborschrank mit zugehörigen Kabel (Gut/Schlechtteile noch aufteile und dazulegen)</t>
+  </si>
+  <si>
+    <t>Ersatzteilkiste</t>
+  </si>
+  <si>
+    <t>Am Ende alles in eine Kiste</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -684,13 +753,31 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="4">
@@ -741,7 +828,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -787,6 +874,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1046,8 +1139,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabelle1" displayName="Tabelle1" ref="A1:I75" totalsRowShown="0">
-  <autoFilter ref="A1:I75" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabelle1" displayName="Tabelle1" ref="A1:I78" totalsRowShown="0">
+  <autoFilter ref="A1:I78" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Nr."/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Thema"/>
@@ -1245,7 +1338,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I81"/>
+  <dimension ref="A1:I85"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.140625" customWidth="1"/>
@@ -1256,7 +1349,7 @@
     <col min="6" max="6" width="9.85546875" customWidth="1"/>
     <col min="7" max="7" width="9.140625" style="1"/>
     <col min="8" max="8" width="13.140625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="84.7109375" customWidth="1"/>
+    <col min="9" max="9" width="97.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1363,7 +1456,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1377,7 +1470,7 @@
         <v>23</v>
       </c>
       <c r="E5" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F5">
         <v>3</v>
@@ -1385,8 +1478,8 @@
       <c r="H5" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="I5" t="s">
-        <v>25</v>
+      <c r="I5" s="6" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -1394,10 +1487,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" t="s">
         <v>26</v>
-      </c>
-      <c r="C6" t="s">
-        <v>27</v>
       </c>
       <c r="D6" t="s">
         <v>11</v>
@@ -1412,7 +1505,7 @@
         <v>13</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -1420,16 +1513,16 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" t="s">
         <v>30</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
         <v>31</v>
-      </c>
-      <c r="D7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" t="s">
-        <v>32</v>
       </c>
       <c r="F7">
         <v>1</v>
@@ -1438,7 +1531,7 @@
         <v>13</v>
       </c>
       <c r="I7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -1446,10 +1539,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" t="s">
         <v>34</v>
-      </c>
-      <c r="C8" t="s">
-        <v>35</v>
       </c>
       <c r="D8" t="s">
         <v>11</v>
@@ -1469,16 +1562,16 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" t="s">
         <v>36</v>
       </c>
-      <c r="C9" t="s">
-        <v>37</v>
-      </c>
       <c r="D9" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="E9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F9">
         <v>2</v>
@@ -1487,7 +1580,7 @@
         <v>13</v>
       </c>
       <c r="I9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -1495,10 +1588,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" t="s">
         <v>39</v>
-      </c>
-      <c r="C10" t="s">
-        <v>40</v>
       </c>
       <c r="D10" t="s">
         <v>11</v>
@@ -1513,7 +1606,7 @@
         <v>13</v>
       </c>
       <c r="I10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -1521,10 +1614,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" t="s">
         <v>42</v>
-      </c>
-      <c r="C11" t="s">
-        <v>43</v>
       </c>
       <c r="D11" t="s">
         <v>11</v>
@@ -1544,10 +1637,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C12" t="s">
         <v>44</v>
-      </c>
-      <c r="C12" t="s">
-        <v>45</v>
       </c>
       <c r="D12" t="s">
         <v>11</v>
@@ -1562,7 +1655,7 @@
         <v>13</v>
       </c>
       <c r="I12" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -1570,10 +1663,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
+        <v>46</v>
+      </c>
+      <c r="C13" t="s">
         <v>47</v>
-      </c>
-      <c r="C13" t="s">
-        <v>48</v>
       </c>
       <c r="D13" t="s">
         <v>11</v>
@@ -1593,10 +1686,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
+        <v>48</v>
+      </c>
+      <c r="C14" t="s">
         <v>49</v>
-      </c>
-      <c r="C14" t="s">
-        <v>50</v>
       </c>
       <c r="D14" t="s">
         <v>11</v>
@@ -1616,10 +1709,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
+        <v>50</v>
+      </c>
+      <c r="C15" t="s">
         <v>51</v>
-      </c>
-      <c r="C15" t="s">
-        <v>52</v>
       </c>
       <c r="D15" t="s">
         <v>11</v>
@@ -1634,7 +1727,7 @@
         <v>13</v>
       </c>
       <c r="I15" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -1642,13 +1735,13 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
+        <v>53</v>
+      </c>
+      <c r="C16" t="s">
         <v>54</v>
       </c>
-      <c r="C16" t="s">
-        <v>55</v>
-      </c>
       <c r="D16" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="E16" t="s">
         <v>24</v>
@@ -1658,6 +1751,9 @@
       </c>
       <c r="G16" s="1" t="s">
         <v>13</v>
+      </c>
+      <c r="I16" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -1665,10 +1761,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C17" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D17" t="s">
         <v>11</v>
@@ -1688,10 +1784,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
+        <v>56</v>
+      </c>
+      <c r="C18" t="s">
         <v>57</v>
-      </c>
-      <c r="C18" t="s">
-        <v>58</v>
       </c>
       <c r="D18" t="s">
         <v>11</v>
@@ -1711,16 +1807,16 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
+        <v>58</v>
+      </c>
+      <c r="C19" t="s">
         <v>59</v>
       </c>
-      <c r="C19" t="s">
-        <v>60</v>
-      </c>
       <c r="D19" t="s">
         <v>11</v>
       </c>
       <c r="E19" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F19">
         <v>3</v>
@@ -1729,7 +1825,7 @@
         <v>13</v>
       </c>
       <c r="I19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -1737,10 +1833,10 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
+        <v>61</v>
+      </c>
+      <c r="C20" t="s">
         <v>62</v>
-      </c>
-      <c r="C20" t="s">
-        <v>63</v>
       </c>
       <c r="D20" t="s">
         <v>11</v>
@@ -1755,7 +1851,7 @@
         <v>13</v>
       </c>
       <c r="I20" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
@@ -1763,16 +1859,16 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
+        <v>64</v>
+      </c>
+      <c r="C21" t="s">
         <v>65</v>
       </c>
-      <c r="C21" t="s">
-        <v>66</v>
-      </c>
       <c r="D21" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="E21" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F21">
         <v>2</v>
@@ -1786,10 +1882,10 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
+        <v>66</v>
+      </c>
+      <c r="C22" t="s">
         <v>67</v>
-      </c>
-      <c r="C22" t="s">
-        <v>68</v>
       </c>
       <c r="D22" t="s">
         <v>11</v>
@@ -1801,10 +1897,10 @@
         <v>1</v>
       </c>
       <c r="G22" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="I22" t="s">
         <v>69</v>
-      </c>
-      <c r="I22" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -1812,10 +1908,10 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
+        <v>70</v>
+      </c>
+      <c r="C23" t="s">
         <v>71</v>
-      </c>
-      <c r="C23" t="s">
-        <v>72</v>
       </c>
       <c r="D23" t="s">
         <v>11</v>
@@ -1827,10 +1923,10 @@
         <v>1</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I23" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -1838,10 +1934,10 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
+        <v>73</v>
+      </c>
+      <c r="C24" t="s">
         <v>74</v>
-      </c>
-      <c r="C24" t="s">
-        <v>75</v>
       </c>
       <c r="D24" t="s">
         <v>11</v>
@@ -1853,15 +1949,18 @@
         <v>3</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I24" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" s="8" t="s">
         <v>76</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B25" s="8" t="s">
-        <v>77</v>
       </c>
       <c r="C25" s="8"/>
       <c r="D25" t="s">
@@ -1876,13 +1975,13 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B26" t="s">
+        <v>77</v>
+      </c>
+      <c r="C26" t="s">
         <v>78</v>
-      </c>
-      <c r="C26" t="s">
-        <v>79</v>
       </c>
       <c r="D26" t="s">
         <v>11</v>
@@ -1894,18 +1993,18 @@
         <v>2</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C27" t="s">
-        <v>199</v>
+        <v>190</v>
       </c>
       <c r="D27" t="s">
         <v>11</v>
@@ -1917,18 +2016,18 @@
         <v>3</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C28" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="D28" t="s">
         <v>11</v>
@@ -1940,18 +2039,18 @@
         <v>1</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B29" t="s">
+        <v>81</v>
+      </c>
+      <c r="C29" t="s">
         <v>82</v>
-      </c>
-      <c r="C29" t="s">
-        <v>83</v>
       </c>
       <c r="D29" t="s">
         <v>11</v>
@@ -1963,18 +2062,18 @@
         <v>1</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C30" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="D30" t="s">
         <v>11</v>
@@ -1986,18 +2085,18 @@
         <v>1</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C31" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="D31" t="s">
         <v>11</v>
@@ -2009,18 +2108,18 @@
         <v>1</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C32" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="D32" t="s">
         <v>11</v>
@@ -2032,18 +2131,18 @@
         <v>1</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C33" t="s">
-        <v>199</v>
+        <v>190</v>
       </c>
       <c r="D33" t="s">
         <v>11</v>
@@ -2055,285 +2154,291 @@
         <v>3</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>33</v>
+      </c>
       <c r="B34" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C34" s="9"/>
       <c r="D34" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E34" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F34">
         <v>1</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B35" t="s">
+        <v>89</v>
+      </c>
+      <c r="C35" t="s">
         <v>90</v>
       </c>
-      <c r="C35" t="s">
-        <v>91</v>
-      </c>
       <c r="D35" t="s">
         <v>11</v>
       </c>
       <c r="E35" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F35">
         <v>1</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B36" t="s">
+        <v>91</v>
+      </c>
+      <c r="C36" t="s">
         <v>92</v>
       </c>
-      <c r="C36" t="s">
-        <v>93</v>
-      </c>
       <c r="D36" t="s">
         <v>11</v>
       </c>
       <c r="E36" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F36">
         <v>1</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B37" t="s">
+        <v>93</v>
+      </c>
+      <c r="C37" t="s">
         <v>94</v>
       </c>
-      <c r="C37" t="s">
-        <v>95</v>
-      </c>
       <c r="D37" t="s">
         <v>11</v>
       </c>
       <c r="E37" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F37">
         <v>1</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C38" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D38" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E38" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F38">
         <v>2</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B39" t="s">
+        <v>96</v>
+      </c>
+      <c r="C39" t="s">
         <v>97</v>
       </c>
-      <c r="C39" t="s">
-        <v>98</v>
-      </c>
       <c r="D39" t="s">
         <v>11</v>
       </c>
       <c r="E39" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F39">
         <v>2</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B40" t="s">
+        <v>98</v>
+      </c>
+      <c r="C40" t="s">
+        <v>97</v>
+      </c>
+      <c r="D40" t="s">
+        <v>11</v>
+      </c>
+      <c r="E40" t="s">
+        <v>31</v>
+      </c>
+      <c r="F40">
+        <v>2</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41" s="8" t="s">
         <v>99</v>
-      </c>
-      <c r="C40" t="s">
-        <v>98</v>
-      </c>
-      <c r="D40" t="s">
-        <v>11</v>
-      </c>
-      <c r="E40" t="s">
-        <v>32</v>
-      </c>
-      <c r="F40">
-        <v>2</v>
-      </c>
-      <c r="G40" s="1" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B41" s="8" t="s">
-        <v>100</v>
       </c>
       <c r="C41" s="8"/>
       <c r="D41" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E41" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F41">
         <v>2</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B42" t="s">
+        <v>100</v>
+      </c>
+      <c r="C42" t="s">
         <v>101</v>
       </c>
-      <c r="C42" t="s">
-        <v>102</v>
-      </c>
       <c r="D42" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="E42" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F42">
         <v>2</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B43" t="s">
+        <v>102</v>
+      </c>
+      <c r="C43" t="s">
         <v>103</v>
       </c>
-      <c r="C43" t="s">
-        <v>104</v>
-      </c>
       <c r="D43" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="E43" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F43">
         <v>2</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B44" t="s">
+        <v>104</v>
+      </c>
+      <c r="C44" t="s">
         <v>105</v>
       </c>
-      <c r="C44" t="s">
-        <v>106</v>
-      </c>
       <c r="D44" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="E44" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F44">
         <v>2</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B45" t="s">
+        <v>106</v>
+      </c>
+      <c r="C45" t="s">
         <v>107</v>
       </c>
-      <c r="C45" t="s">
-        <v>108</v>
-      </c>
       <c r="D45" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E45" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F45">
         <v>2</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B46" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C46" s="8"/>
       <c r="D46" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E46" t="s">
         <v>17</v>
@@ -2342,41 +2447,44 @@
         <v>1</v>
       </c>
       <c r="G46" s="1" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A47">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B47" t="s">
+        <v>109</v>
+      </c>
+      <c r="C47" t="s">
         <v>110</v>
       </c>
-      <c r="C47" t="s">
+      <c r="D47" t="s">
+        <v>27</v>
+      </c>
+      <c r="E47" t="s">
+        <v>208</v>
+      </c>
+      <c r="F47">
+        <v>1</v>
+      </c>
+      <c r="G47" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="I47" s="18" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48" t="s">
         <v>111</v>
       </c>
-      <c r="D47" t="s">
-        <v>23</v>
-      </c>
-      <c r="E47" t="s">
-        <v>17</v>
-      </c>
-      <c r="F47">
-        <v>1</v>
-      </c>
-      <c r="G47" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="I47" s="6" t="s">
+      <c r="C48" t="s">
         <v>112</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B48" t="s">
-        <v>113</v>
-      </c>
-      <c r="C48" t="s">
-        <v>114</v>
       </c>
       <c r="D48" t="s">
         <v>11</v>
@@ -2388,18 +2496,18 @@
         <v>2</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C49" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D49" t="s">
         <v>11</v>
@@ -2411,18 +2519,18 @@
         <v>2</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="50" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A50">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B50" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C50" s="11" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D50" s="10" t="s">
         <v>11</v>
@@ -2434,21 +2542,21 @@
         <v>1</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B51" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C51" s="11" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D51" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="E51" s="10" t="s">
         <v>17</v>
@@ -2457,18 +2565,18 @@
         <v>1</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B52" s="10" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C52" s="11" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D52" t="s">
         <v>11</v>
@@ -2480,21 +2588,21 @@
         <v>1</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I52" s="10" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="53" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A53">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B53" s="10" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C53" s="11" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D53" t="s">
         <v>11</v>
@@ -2506,48 +2614,48 @@
         <v>1</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I53" s="10"/>
     </row>
     <row r="54" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A54">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B54" s="10" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C54" s="11" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D54" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="E54" s="10" t="s">
-        <v>128</v>
+        <v>12</v>
       </c>
       <c r="F54" s="10">
         <v>3</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I54" s="10" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="C55" s="11" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="55" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A55">
-        <v>50</v>
-      </c>
-      <c r="B55" s="10" t="s">
-        <v>130</v>
-      </c>
-      <c r="C55" s="11" t="s">
-        <v>131</v>
-      </c>
       <c r="D55" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E55" s="10" t="s">
         <v>12</v>
@@ -2556,21 +2664,21 @@
         <v>2</v>
       </c>
       <c r="H55" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="I55" s="10" t="s">
-        <v>132</v>
+        <v>68</v>
+      </c>
+      <c r="I55" s="11" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="56" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A56">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B56" s="10" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C56" s="11" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="D56" t="s">
         <v>11</v>
@@ -2582,21 +2690,21 @@
         <v>1</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I56" s="10" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B57" s="10" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C57" s="11" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="D57" t="s">
         <v>11</v>
@@ -2608,24 +2716,24 @@
         <v>3</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I57" s="10" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="58" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A58">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B58" s="10" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C58" s="10" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="D58" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>12</v>
@@ -2634,21 +2742,21 @@
         <v>2</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="I58" s="11" t="s">
-        <v>200</v>
+        <v>68</v>
+      </c>
+      <c r="I58" s="19" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="B59" s="10" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="C59" s="11" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="D59" t="s">
         <v>11</v>
@@ -2660,24 +2768,24 @@
         <v>2</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I59" s="10" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A60">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B60" s="10" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C60" s="11" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="D60" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="E60" s="10" t="s">
         <v>17</v>
@@ -2686,44 +2794,44 @@
         <v>2</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I60" s="11" t="s">
-        <v>146</v>
+        <v>197</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="B61" s="10" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="C61" s="11" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="D61" t="s">
         <v>11</v>
       </c>
       <c r="E61" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F61" s="10">
         <v>3</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B62" s="10" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="C62" s="11" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="D62" t="s">
         <v>11</v>
@@ -2735,135 +2843,135 @@
         <v>2</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B63" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="C63" s="11" t="s">
+        <v>148</v>
+      </c>
+      <c r="D63" t="s">
+        <v>27</v>
+      </c>
+      <c r="E63" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="F63" s="10">
+        <v>1</v>
+      </c>
+      <c r="G63" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="I63" s="7" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>63</v>
+      </c>
+      <c r="B64" s="10" t="s">
         <v>151</v>
-      </c>
-      <c r="C63" s="11" t="s">
-        <v>152</v>
-      </c>
-      <c r="D63" t="s">
-        <v>28</v>
-      </c>
-      <c r="E63" s="10" t="s">
-        <v>153</v>
-      </c>
-      <c r="F63" s="10">
-        <v>1</v>
-      </c>
-      <c r="G63" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="I63" s="7" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="64" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A64">
-        <v>59</v>
-      </c>
-      <c r="B64" s="10" t="s">
-        <v>155</v>
       </c>
       <c r="C64" s="11"/>
       <c r="D64" t="s">
         <v>23</v>
       </c>
       <c r="E64" s="10" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F64" s="10">
         <v>3</v>
       </c>
       <c r="H64" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I64" s="12" t="s">
-        <v>156</v>
+        <v>198</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B65" s="10" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="C65" s="11"/>
       <c r="D65" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E65" s="10" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="F65" s="10">
         <v>1</v>
       </c>
       <c r="G65" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="66" spans="1:9" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A66">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B66" s="13" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C66" s="11" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="D66" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E66" s="10" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="F66" s="10">
         <v>1</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I66" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="B67" s="8" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="D67" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="E67" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="F67">
         <v>2</v>
       </c>
       <c r="G67" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B68" s="10" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="C68" s="11" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="D68" t="s">
         <v>11</v>
@@ -2875,21 +2983,21 @@
         <v>2</v>
       </c>
       <c r="G68" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I68" s="10" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B69" s="10" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="C69" s="11" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="D69" t="s">
         <v>11</v>
@@ -2901,45 +3009,45 @@
         <v>2</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I69" s="10" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B70" s="10" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="C70" s="11" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="D70" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="E70" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F70" s="10">
         <v>2</v>
       </c>
       <c r="G70" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I70" s="10"/>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B71" s="10" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="C71" s="11" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="D71" t="s">
         <v>11</v>
@@ -2951,137 +3059,197 @@
         <v>3</v>
       </c>
       <c r="G71" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I71" s="10"/>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B72" s="10" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="C72" s="11" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="D72" t="s">
         <v>23</v>
       </c>
       <c r="E72" s="10" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F72" s="10"/>
       <c r="H72" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I72" s="10" t="s">
-        <v>174</v>
+        <v>199</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B73" s="10" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C73" s="11" t="s">
-        <v>176</v>
+        <v>139</v>
       </c>
       <c r="D73" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="E73" s="10" t="s">
-        <v>177</v>
+        <v>12</v>
       </c>
       <c r="F73" s="10">
         <v>2</v>
       </c>
-      <c r="H73" s="1" t="s">
-        <v>69</v>
+      <c r="G73" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="I73" s="10" t="s">
-        <v>132</v>
+        <v>174</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74">
-        <v>69</v>
-      </c>
-      <c r="B74" s="10" t="s">
-        <v>178</v>
-      </c>
-      <c r="C74" s="11" t="s">
-        <v>142</v>
+        <v>73</v>
+      </c>
+      <c r="B74" t="s">
+        <v>191</v>
+      </c>
+      <c r="C74" t="s">
+        <v>192</v>
       </c>
       <c r="D74" t="s">
-        <v>11</v>
-      </c>
-      <c r="E74" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="F74" s="10">
-        <v>2</v>
+        <v>27</v>
+      </c>
+      <c r="E74" t="s">
+        <v>153</v>
+      </c>
+      <c r="F74">
+        <v>1</v>
       </c>
       <c r="G74" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="I74" s="10" t="s">
-        <v>179</v>
+        <v>68</v>
+      </c>
+      <c r="I74" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B75" t="s">
+        <v>200</v>
+      </c>
+      <c r="C75" t="s">
         <v>201</v>
       </c>
-      <c r="C75" t="s">
+      <c r="D75" t="s">
+        <v>27</v>
+      </c>
+      <c r="E75" t="s">
+        <v>12</v>
+      </c>
+      <c r="F75">
+        <v>1</v>
+      </c>
+      <c r="G75" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A76">
+        <v>75</v>
+      </c>
+      <c r="B76" t="s">
         <v>202</v>
       </c>
-      <c r="D75" t="s">
+      <c r="C76" t="s">
+        <v>203</v>
+      </c>
+      <c r="D76" t="s">
         <v>23</v>
       </c>
-      <c r="E75" t="s">
-        <v>158</v>
+      <c r="E76" t="s">
+        <v>153</v>
+      </c>
+      <c r="F76">
+        <v>2</v>
+      </c>
+      <c r="G76" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A77">
+        <v>76</v>
+      </c>
+      <c r="B77" t="s">
+        <v>213</v>
+      </c>
+      <c r="C77" t="s">
+        <v>204</v>
+      </c>
+      <c r="D77" t="s">
+        <v>23</v>
+      </c>
+      <c r="E77" t="s">
+        <v>153</v>
+      </c>
+      <c r="F77">
+        <v>2</v>
+      </c>
+      <c r="G77" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="I77" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A78">
+        <v>77</v>
+      </c>
       <c r="B78" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
       <c r="C78" t="s">
+        <v>206</v>
+      </c>
+      <c r="D78" t="s">
+        <v>27</v>
+      </c>
+      <c r="E78" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B79" t="s">
-        <v>181</v>
-      </c>
-      <c r="C79" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B80" t="s">
-        <v>182</v>
-      </c>
-      <c r="C80" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="81" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B81" t="s">
-        <v>183</v>
-      </c>
-      <c r="C81" t="s">
-        <v>24</v>
+      <c r="F78">
+        <v>1</v>
+      </c>
+      <c r="G78" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="85" spans="2:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="B85" t="s">
+        <v>209</v>
+      </c>
+      <c r="C85" t="s">
+        <v>153</v>
+      </c>
+      <c r="D85" t="s">
+        <v>177</v>
+      </c>
+      <c r="I85" s="18" t="s">
+        <v>210</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="D2:D75">
+  <conditionalFormatting sqref="D2:D78">
     <cfRule type="cellIs" dxfId="15" priority="8" operator="equal">
       <formula>"Not started"</formula>
     </cfRule>
@@ -3092,7 +3260,7 @@
       <formula>"Done"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E75">
+  <conditionalFormatting sqref="E2:E78">
     <cfRule type="containsText" dxfId="12" priority="2" operator="containsText" text="Alle">
       <formula>NOT(ISERROR(SEARCH("Alle",E2)))</formula>
     </cfRule>
@@ -3137,7 +3305,7 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>184</v>
+        <v>175</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -3160,7 +3328,7 @@
         <v>5</v>
       </c>
       <c r="G2" s="17" t="s">
-        <v>185</v>
+        <v>176</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="45" x14ac:dyDescent="0.25">
@@ -3168,16 +3336,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
       <c r="F3" s="10">
         <v>1</v>
@@ -3188,16 +3356,16 @@
         <v>2</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
       <c r="F4" s="10">
         <v>1</v>
@@ -3208,22 +3376,22 @@
         <v>3</v>
       </c>
       <c r="B5" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>178</v>
+      </c>
+      <c r="F5" s="10">
+        <v>1</v>
+      </c>
+      <c r="G5" s="10" t="s">
         <v>121</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>122</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>190</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>187</v>
-      </c>
-      <c r="F5" s="10">
-        <v>1</v>
-      </c>
-      <c r="G5" s="10" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="45" x14ac:dyDescent="0.25">
@@ -3231,13 +3399,13 @@
         <v>4</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
       <c r="F6" s="10">
         <v>1</v>
@@ -3248,19 +3416,19 @@
         <v>5</v>
       </c>
       <c r="B7" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="E7" s="10" t="s">
         <v>126</v>
-      </c>
-      <c r="C7" s="11" t="s">
-        <v>127</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>128</v>
       </c>
       <c r="F7" s="10">
         <v>3</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="45" x14ac:dyDescent="0.25">
@@ -3268,19 +3436,19 @@
         <v>6</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F8" s="10">
         <v>2</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="45" x14ac:dyDescent="0.25">
@@ -3288,19 +3456,19 @@
         <v>7</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
       <c r="F9" s="10">
         <v>1</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -3308,10 +3476,10 @@
         <v>8</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>12</v>
@@ -3320,7 +3488,7 @@
         <v>3</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -3328,10 +3496,10 @@
         <v>9</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>12</v>
@@ -3340,7 +3508,7 @@
         <v>2</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -3348,10 +3516,10 @@
         <v>10</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="E12" s="10" t="s">
         <v>12</v>
@@ -3360,7 +3528,7 @@
         <v>2</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>195</v>
+        <v>186</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="30" x14ac:dyDescent="0.25">
@@ -3368,19 +3536,19 @@
         <v>11</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E13" s="10" t="s">
+        <v>178</v>
+      </c>
+      <c r="F13" s="10">
+        <v>2</v>
+      </c>
+      <c r="G13" s="10" t="s">
         <v>187</v>
-      </c>
-      <c r="F13" s="10">
-        <v>2</v>
-      </c>
-      <c r="G13" s="10" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="30" x14ac:dyDescent="0.25">
@@ -3388,13 +3556,13 @@
         <v>12</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F14" s="10">
         <v>3</v>
@@ -3405,10 +3573,10 @@
         <v>13</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E15" s="10" t="s">
         <v>24</v>
@@ -3422,13 +3590,13 @@
         <v>14</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="F16" s="10">
         <v>1</v>
@@ -3439,10 +3607,10 @@
         <v>15</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F17" s="10">
         <v>3</v>
@@ -3450,10 +3618,10 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B18" s="10" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="F18" s="10">
         <v>1</v>
@@ -3461,13 +3629,13 @@
     </row>
     <row r="19" spans="1:7" ht="30.75" x14ac:dyDescent="0.3">
       <c r="B19" s="13" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="F19" s="10">
         <v>1</v>
@@ -3475,7 +3643,7 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="10" t="s">
-        <v>197</v>
+        <v>188</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -3498,7 +3666,7 @@
         <v>5</v>
       </c>
       <c r="G23" s="17" t="s">
-        <v>185</v>
+        <v>176</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="30" x14ac:dyDescent="0.25">
@@ -3506,19 +3674,19 @@
         <v>1</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F24" s="10">
         <v>2</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="30" x14ac:dyDescent="0.25">
@@ -3526,13 +3694,13 @@
         <v>2</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F25" s="10">
         <v>2</v>
@@ -3543,13 +3711,13 @@
         <v>3</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F26" s="10">
         <v>2</v>
@@ -3560,10 +3728,10 @@
         <v>4</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="E27" s="10" t="s">
         <v>24</v>
@@ -3577,16 +3745,16 @@
         <v>5</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="30" x14ac:dyDescent="0.25">
@@ -3594,19 +3762,19 @@
         <v>6</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="F29" s="10">
         <v>2</v>
       </c>
       <c r="G29" s="10" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
@@ -3614,10 +3782,10 @@
         <v>7</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="E30" s="10" t="s">
         <v>12</v>

</xml_diff>